<commit_message>
Rich agent answers, thinking bubble, library-access intent, variable-length docs, demote duplicate copies
- Agent: library-access handler reads real library permissions; Markdown-rich answers rendered safely in the UI; animated thinking bubble
- Foundry agent instructions: use live evidence for governance questions, rich Markdown format
- Corpus: random (stable) page/slide/sheet counts; copies seeded as Draft duplicates of approved originals
- Fix agent provisioning: keep governance source fields, multi-hub smoke test
- Refresh screenshots, agent test and READMEs

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/sites/hr/Employee Relations/employee-relations-case-tracker.xlsx
+++ b/data/sites/hr/Employee Relations/employee-relations-case-tracker.xlsx
@@ -14,11 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 RACI Matrix" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Procedures" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Risk Register" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Quality Audit" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Escalations" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 SLAs" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Roadmap" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Sign-off" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Sign-off" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -250,66 +246,6 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="4572000" cy="1524000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="4572000" cy="1524000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -789,559 +725,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Employee Relations Case Tracker - Section 10: Cross-Functional Dependencies</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>HR Knowledge Hub | Employee Relations | Owner: Ben Okafor  |  Last updated: October 30, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Log of open and closed employee relations cases with case type, status, and days open, used to monitor caseload and resolution time. Section 10 (Cross-Functional Dependencies) applies to Employee Relations within HR Knowledge Hub and is maintained by Ben Okafor. Documents upstream and downstream team dependencies and service-level commitments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Operational requirement 10.1: Cases open longer than 20 business days are escalated to the VP of People. Secondary control 10.2: Case types include conduct, performance, accommodation, and harassment complaints.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Case Type</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Days Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Conduct</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Accommodation</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Performance</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Harassment Complaint</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Sec-10</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Stage 10 Verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Governance Checkpoints</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>• Cases open longer than 20 business days are escalated to the VP of People.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>• Case types include conduct, performance, accommodation, and harassment complaints.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>• Section 10 review cadence is tracked by Ben Okafor under Employee Relations governance.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Employee Relations Case Tracker - Section 11: Continuous Improvement Roadmap</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>HR Knowledge Hub | Employee Relations | Owner: Ben Okafor  |  Last updated: October 30, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Log of open and closed employee relations cases with case type, status, and days open, used to monitor caseload and resolution time. Section 11 (Continuous Improvement Roadmap) applies to Employee Relations within HR Knowledge Hub and is maintained by Ben Okafor. Schedules quarterly optimization milestones, automation targets, and capability reviews.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Operational requirement 11.1: Case types include conduct, performance, accommodation, and harassment complaints. Secondary control 11.2: All case notes are stored in the restricted Employee Relations case file, not this tracker.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Case Type</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Days Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Conduct</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Accommodation</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Performance</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Harassment Complaint</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Sec-11</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Stage 11 Verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Governance Checkpoints</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>• Case types include conduct, performance, accommodation, and harassment complaints.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>• All case notes are stored in the restricted Employee Relations case file, not this tracker.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>• Section 11 review cadence is tracked by Ben Okafor under Employee Relations governance.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Employee Relations Case Tracker - Section 12: Appendix, Lineage &amp; Sign-off</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>HR Knowledge Hub | Employee Relations | Owner: Ben Okafor  |  Last updated: October 30, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Log of open and closed employee relations cases with case type, status, and days open, used to monitor caseload and resolution time. Section 12 (Appendix, Lineage &amp; Sign-off) applies to Employee Relations within HR Knowledge Hub and is maintained by Ben Okafor. Records document lineage, governance metadata, version history, and owner sign-off.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Operational requirement 12.1: All case notes are stored in the restricted Employee Relations case file, not this tracker. Secondary control 12.2: Average case resolution time target is 10 business days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Case Type</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Days Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Conduct</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Accommodation</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Performance</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Harassment Complaint</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Sec-12</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Stage 12 Verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Governance Checkpoints</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>• All case notes are stored in the restricted Employee Relations case file, not this tracker.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>• Average case resolution time target is 10 business days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>• Section 12 review cadence is tracked by Ben Okafor under Employee Relations governance.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2467,7 +1850,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Employee Relations Case Tracker - Section 8: Quality Assurance &amp; Audits</t>
+          <t>Employee Relations Case Tracker - Section 8: Appendix, Lineage &amp; Sign-off</t>
         </is>
       </c>
     </row>
@@ -2481,7 +1864,7 @@
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Log of open and closed employee relations cases with case type, status, and days open, used to monitor caseload and resolution time. Section 8 (Quality Assurance &amp; Audits) applies to Employee Relations within HR Knowledge Hub and is maintained by Ben Okafor. Specifies sampling frequencies, inspection tolerances, and nonconformance workflows.</t>
+          <t>Log of open and closed employee relations cases with case type, status, and days open, used to monitor caseload and resolution time. Section 8 (Appendix, Lineage &amp; Sign-off) applies to Employee Relations within HR Knowledge Hub and is maintained by Ben Okafor. Records document lineage, governance metadata, version history, and owner sign-off.</t>
         </is>
       </c>
     </row>
@@ -2619,191 +2002,6 @@
       <c r="A16" t="inlineStr">
         <is>
           <t>• Section 8 review cadence is tracked by Ben Okafor under Employee Relations governance.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Employee Relations Case Tracker - Section 9: Exception Handling &amp; Escalations</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>HR Knowledge Hub | Employee Relations | Owner: Ben Okafor  |  Last updated: October 30, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Log of open and closed employee relations cases with case type, status, and days open, used to monitor caseload and resolution time. Section 9 (Exception Handling &amp; Escalations) applies to Employee Relations within HR Knowledge Hub and is maintained by Ben Okafor. Outlines severity tiers, response SLAs, and cross-functional escalation paths.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Operational requirement 9.1: Average case resolution time target is 10 business days. Secondary control 9.2: Cases open longer than 20 business days are escalated to the VP of People.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Case Type</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Days Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Conduct</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Accommodation</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Performance</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Harassment Complaint</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Sec-9</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Stage 9 Verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Governance Checkpoints</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>• Average case resolution time target is 10 business days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>• Cases open longer than 20 business days are escalated to the VP of People.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>• Section 9 review cadence is tracked by Ben Okafor under Employee Relations governance.</t>
         </is>
       </c>
     </row>

</xml_diff>